<commit_message>
fix: count Dec 2010 orders once; redesign the live dashboard
- prepare_real_data: the source workbook's two yearly sheets overlap on
  1-9 Dec 2010. Reading both doubled those 776 orders (revenue +1.8%).
  Each invoice is now read once; a test fails if the window looks doubled.
- crm_retention: months the data does not fully cover are null, not 0%
  (late cohorts are right-censored); notebook cross-check updated.
- build_web_dashboard: rebuilt page with HTML/CSS charts, takeaways, all
  25 cohorts, CLV decomposition, A/B confidence interval, mobile layout
  and a social preview image.
- build_summary reuses the zero-safe deep-dive helpers; every output is
  written with LF so Windows runs leave a clean tree.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/crm_dashboard.xlsx
+++ b/dashboard/crm_dashboard.xlsx
@@ -467,13 +467,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1532</v>
+        <v>1537</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2606</v>
+        <v>0.2615</v>
       </c>
       <c r="D2" t="n">
-        <v>12662714.43</v>
+        <v>12433252.98</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -493,13 +493,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1596</v>
+        <v>0.1594</v>
       </c>
       <c r="D3" t="n">
-        <v>2310803.78</v>
+        <v>2283898.41</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -525,7 +525,7 @@
         <v>0.1997</v>
       </c>
       <c r="D4" t="n">
-        <v>1449812.55</v>
+        <v>1402158.49</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -545,13 +545,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1803</v>
+        <v>0.1802</v>
       </c>
       <c r="D5" t="n">
-        <v>462962.76</v>
+        <v>461722.15</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -571,13 +571,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0201</v>
+        <v>0.0202</v>
       </c>
       <c r="D6" t="n">
-        <v>390847.15</v>
+        <v>392087.76</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -597,13 +597,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0994</v>
+        <v>0.0988</v>
       </c>
       <c r="D7" t="n">
-        <v>258364.15</v>
+        <v>251782.86</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -623,13 +623,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0803</v>
+        <v>0.0801</v>
       </c>
       <c r="D8" t="n">
-        <v>207924.34</v>
+        <v>206648.51</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -696,10 +696,10 @@
         <v>7.38</v>
       </c>
       <c r="D2" t="n">
-        <v>547.0700000000001</v>
+        <v>539.87</v>
       </c>
       <c r="E2" t="n">
-        <v>4039.09</v>
+        <v>3985.97</v>
       </c>
     </row>
     <row r="3">
@@ -715,10 +715,10 @@
         <v>6.56</v>
       </c>
       <c r="D3" t="n">
-        <v>579.64</v>
+        <v>569.33</v>
       </c>
       <c r="E3" t="n">
-        <v>3801.93</v>
+        <v>3734.29</v>
       </c>
     </row>
     <row r="4">
@@ -734,10 +734,10 @@
         <v>3.87</v>
       </c>
       <c r="D4" t="n">
-        <v>718.74</v>
+        <v>713.48</v>
       </c>
       <c r="E4" t="n">
-        <v>2782.83</v>
+        <v>2762.45</v>
       </c>
     </row>
     <row r="5">
@@ -753,10 +753,10 @@
         <v>6.27</v>
       </c>
       <c r="D5" t="n">
-        <v>438.96</v>
+        <v>430.66</v>
       </c>
       <c r="E5" t="n">
-        <v>2752.37</v>
+        <v>2700.27</v>
       </c>
     </row>
   </sheetData>
@@ -1405,9 +1405,6 @@
       <c r="H20" t="n">
         <v>0.287</v>
       </c>
-      <c r="I20" t="n">
-        <v>0.0833</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1433,12 +1430,6 @@
       <c r="G21" t="n">
         <v>0.3431</v>
       </c>
-      <c r="H21" t="n">
-        <v>0.1569</v>
-      </c>
-      <c r="I21" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1461,15 +1452,6 @@
       <c r="F22" t="n">
         <v>0.2642</v>
       </c>
-      <c r="G22" t="n">
-        <v>0.1698</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1489,18 +1471,6 @@
       <c r="E23" t="n">
         <v>0.3757</v>
       </c>
-      <c r="F23" t="n">
-        <v>0.1481</v>
-      </c>
-      <c r="G23" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1517,21 +1487,6 @@
       <c r="D24" t="n">
         <v>0.3213</v>
       </c>
-      <c r="E24" t="n">
-        <v>0.1584</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1545,24 +1500,6 @@
       <c r="C25" t="n">
         <v>1</v>
       </c>
-      <c r="D25" t="n">
-        <v>0.1414</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1575,24 +1512,6 @@
       </c>
       <c r="C26" t="n">
         <v>1</v>
-      </c>
-      <c r="D26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" t="n">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>